<commit_message>
📊 Steam 차트 업데이트: 2026-04-30
</commit_message>
<xml_diff>
--- a/steam_chart_monitor.xlsx
+++ b/steam_chart_monitor.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>642246</v>
+        <v>623143</v>
       </c>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>293667</v>
+        <v>292590</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>178270</v>
+        <v>203712</v>
       </c>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>125283</v>
+        <v>125878</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>120344</v>
+        <v>116307</v>
       </c>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
@@ -851,7 +851,7 @@
         <v/>
       </c>
       <c r="I7" t="n">
-        <v>105719</v>
+        <v>91621</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -902,7 +902,7 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>95183</v>
+        <v>83859</v>
       </c>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
@@ -935,11 +935,11 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>1808500</v>
+        <v>1973530</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ARC Raiders</t>
+          <t>Limbus Company</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -947,31 +947,29 @@
           <t>미확인</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
+      <c r="H9" t="n">
+        <v/>
       </c>
       <c r="I9" t="n">
-        <v>80721</v>
+        <v>79143</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>85.2</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>387404</v>
+        <v>103176</v>
       </c>
       <c r="O9" t="n">
-        <v>58900</v>
+        <v/>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>58900</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -1004,7 +1002,7 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>76045</v>
+        <v>76446</v>
       </c>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
@@ -1037,11 +1035,11 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>3041230</v>
+        <v>2507950</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Windrose</t>
+          <t>Delta Force</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1051,29 +1049,29 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Action, Adventure, RPG, Early Access</t>
+          <t>Action, Adventure, Massively Multiplayer, Free To Play</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>74455</v>
+        <v>74365</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>87.3</v>
+        <v>58.3</v>
       </c>
       <c r="N11" t="n">
-        <v>30189</v>
+        <v>180659</v>
       </c>
       <c r="O11" t="n">
-        <v>32000</v>
+        <v/>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>32000</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1086,11 +1084,11 @@
         <v>11</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>359550</v>
+        <v>1808500</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Tom Clancy's Rainbow Six Siege</t>
+          <t>ARC Raiders</t>
         </is>
       </c>
       <c r="E12" s="2" t="n"/>
@@ -1102,11 +1100,11 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Action, Free To Play</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>67215</v>
+        <v>68747</v>
       </c>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
@@ -1114,19 +1112,19 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>82.5</v>
+        <v>85.2</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>1507511</v>
+        <v>387404</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v/>
+        <v>58900</v>
       </c>
       <c r="P12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v/>
+        <v>58900</v>
       </c>
     </row>
     <row r="13">
@@ -1139,11 +1137,11 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>2507950</v>
+        <v>431960</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Delta Force</t>
+          <t>Wallpaper Engine</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1153,29 +1151,29 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Action, Adventure, Massively Multiplayer, Free To Play</t>
+          <t>Casual, Indie, Animation &amp; Modeling, Design &amp; Illustration, Photo Editing, Utilities</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>66122</v>
+        <v>62641</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>58.3</v>
+        <v>98</v>
       </c>
       <c r="N13" t="n">
-        <v>180659</v>
+        <v>976932</v>
       </c>
       <c r="O13" t="n">
-        <v/>
+        <v>5600</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v/>
+        <v>5600</v>
       </c>
     </row>
     <row r="14">
@@ -1188,11 +1186,11 @@
         <v>13</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>431960</v>
+        <v>3041230</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Wallpaper Engine</t>
+          <t>Windrose</t>
         </is>
       </c>
       <c r="E14" s="2" t="n"/>
@@ -1204,11 +1202,11 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Casual, Indie, Animation &amp; Modeling, Design &amp; Illustration, Photo Editing, Utilities</t>
+          <t>Action, Adventure, RPG, Early Access</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>58572</v>
+        <v>62488</v>
       </c>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
@@ -1216,19 +1214,19 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>98</v>
+        <v>87.3</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>976932</v>
+        <v>30189</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>5600</v>
+        <v>32000</v>
       </c>
       <c r="P14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>5600</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="15">
@@ -1241,11 +1239,11 @@
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>252490</v>
+        <v>359550</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Rust</t>
+          <t>Tom Clancy's Rainbow Six Siege</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1255,29 +1253,29 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Action, Adventure, Indie, Massively Multiplayer, RPG</t>
+          <t>Action, Free To Play</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>54147</v>
+        <v>56454</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>87</v>
+        <v>82.5</v>
       </c>
       <c r="N15" t="n">
-        <v>1353483</v>
+        <v>1507511</v>
       </c>
       <c r="O15" t="n">
-        <v>21000</v>
+        <v/>
       </c>
       <c r="P15" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>42000</v>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1290,11 +1288,11 @@
         <v>15</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2357570</v>
+        <v>252490</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Overwatch®</t>
+          <t>Rust</t>
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
@@ -1306,11 +1304,11 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Action, Free To Play</t>
+          <t>Action, Adventure, Indie, Massively Multiplayer, RPG</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>54073</v>
+        <v>51624</v>
       </c>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
@@ -1318,19 +1316,19 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>29.7</v>
+        <v>87</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>396974</v>
+        <v>1353483</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v/>
+        <v>21000</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v/>
+        <v>42000</v>
       </c>
     </row>
     <row r="17">
@@ -1343,11 +1341,11 @@
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>381210</v>
+        <v>230410</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Dead by Daylight</t>
+          <t>Warframe</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1357,29 +1355,29 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Action, RPG, Free To Play</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>52224</v>
+        <v>49756</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>78.59999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="N17" t="n">
-        <v>893891</v>
+        <v>660361</v>
       </c>
       <c r="O17" t="n">
-        <v>8600</v>
+        <v/>
       </c>
       <c r="P17" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>21500</v>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1392,11 +1390,11 @@
         <v>17</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>230410</v>
+        <v>2357570</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Warframe</t>
+          <t>Overwatch®</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
@@ -1408,11 +1406,11 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Action, RPG, Free To Play</t>
+          <t>Action, Free To Play</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>52143</v>
+        <v>48635</v>
       </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
@@ -1420,10 +1418,10 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>87.7</v>
+        <v>29.7</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>660361</v>
+        <v>396974</v>
       </c>
       <c r="O18" s="2" t="n">
         <v/>
@@ -1445,11 +1443,11 @@
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>3321460</v>
+        <v>381210</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Crimson Desert</t>
+          <t>Dead by Daylight</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1459,29 +1457,29 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Action, Adventure</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>48472</v>
+        <v>46769</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>84</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N19" t="n">
-        <v>143410</v>
+        <v>893891</v>
       </c>
       <c r="O19" t="n">
-        <v>79800</v>
+        <v>8600</v>
       </c>
       <c r="P19" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="Q19" t="n">
-        <v>79800</v>
+        <v>21500</v>
       </c>
     </row>
     <row r="20">
@@ -1494,11 +1492,11 @@
         <v>19</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>553850</v>
+        <v>3321460</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>HELLDIVERS™ 2</t>
+          <t>Crimson Desert</t>
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
@@ -1510,11 +1508,11 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Action, Adventure</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>44924</v>
+        <v>43545</v>
       </c>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
@@ -1522,19 +1520,19 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>76.2</v>
+        <v>84</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>1131669</v>
+        <v>143410</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>44800</v>
+        <v>79800</v>
       </c>
       <c r="P20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>44800</v>
+        <v>79800</v>
       </c>
     </row>
     <row r="21">
@@ -1547,11 +1545,11 @@
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>413150</v>
+        <v>438100</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Stardew Valley</t>
+          <t>VRChat</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1561,29 +1559,29 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Indie, RPG, Simulation</t>
+          <t>Adventure, Casual, Massively Multiplayer, Simulation, Sports, Free To Play, Early Access</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>44500</v>
+        <v>43017</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>98.5</v>
+        <v>75.3</v>
       </c>
       <c r="N21" t="n">
-        <v>1000411</v>
+        <v>261193</v>
       </c>
       <c r="O21" t="n">
-        <v>16000</v>
+        <v/>
       </c>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>16000</v>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1596,11 +1594,11 @@
         <v>21</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>438100</v>
+        <v>413150</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>VRChat</t>
+          <t>Stardew Valley</t>
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
@@ -1612,11 +1610,11 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Adventure, Casual, Massively Multiplayer, Simulation, Sports, Free To Play, Early Access</t>
+          <t>Indie, RPG, Simulation</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>43861</v>
+        <v>41559</v>
       </c>
       <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
@@ -1624,19 +1622,19 @@
         <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>75.3</v>
+        <v>98.5</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>261193</v>
+        <v>1000411</v>
       </c>
       <c r="O22" s="2" t="n">
-        <v/>
+        <v>16000</v>
       </c>
       <c r="P22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q22" s="2" t="n">
-        <v/>
+        <v>16000</v>
       </c>
     </row>
     <row r="23">
@@ -1649,11 +1647,11 @@
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>1973530</v>
+        <v>553850</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Limbus Company</t>
+          <t>HELLDIVERS™ 2</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1661,29 +1659,31 @@
           <t>미확인</t>
         </is>
       </c>
-      <c r="H23" t="n">
-        <v/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
       </c>
       <c r="I23" t="n">
-        <v>43573</v>
+        <v>39047</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>87.59999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="N23" t="n">
-        <v>103176</v>
+        <v>1131669</v>
       </c>
       <c r="O23" t="n">
-        <v/>
+        <v>44800</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v/>
+        <v>44800</v>
       </c>
     </row>
     <row r="24">
@@ -1696,11 +1696,11 @@
         <v>23</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>322170</v>
+        <v>440</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Geometry Dash</t>
+          <t>Team Fortress 2</t>
         </is>
       </c>
       <c r="E24" s="2" t="n"/>
@@ -1712,11 +1712,11 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Action, Indie</t>
+          <t>Action, Free To Play</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>39322</v>
+        <v>35353</v>
       </c>
       <c r="J24" s="2" t="n"/>
       <c r="K24" s="2" t="n"/>
@@ -1724,19 +1724,19 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>93.09999999999999</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>583368</v>
+        <v>1228472</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>5600</v>
+        <v/>
       </c>
       <c r="P24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>5600</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1749,11 +1749,11 @@
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>440</v>
+        <v>322170</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Team Fortress 2</t>
+          <t>Geometry Dash</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1763,29 +1763,29 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Action, Free To Play</t>
+          <t>Action, Indie</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>38874</v>
+        <v>33833</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>90.90000000000001</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="N25" t="n">
-        <v>1228472</v>
+        <v>583368</v>
       </c>
       <c r="O25" t="n">
-        <v/>
+        <v>5600</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v/>
+        <v>5600</v>
       </c>
     </row>
     <row r="26">
@@ -1798,11 +1798,11 @@
         <v>25</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1086940</v>
+        <v>236390</v>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Baldur's Gate 3</t>
+          <t>War Thunder</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
@@ -1814,11 +1814,11 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Adventure, RPG, Strategy</t>
+          <t>Action, Massively Multiplayer, Simulation, Free To Play</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>34920</v>
+        <v>30342</v>
       </c>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
@@ -1826,19 +1826,19 @@
         <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>96.8</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>836348</v>
+        <v>741169</v>
       </c>
       <c r="O26" s="2" t="n">
-        <v>66000</v>
+        <v/>
       </c>
       <c r="P26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>66000</v>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>642246</v>
+        <v>623143</v>
       </c>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
@@ -1994,7 +1994,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>293667</v>
+        <v>292590</v>
       </c>
       <c r="J5" t="n">
         <v>80.90000000000001</v>
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>178270</v>
+        <v>203712</v>
       </c>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="n"/>
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>125283</v>
+        <v>125878</v>
       </c>
       <c r="J7" t="n">
         <v>96.59999999999999</v>
@@ -2096,7 +2096,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>120344</v>
+        <v>116307</v>
       </c>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="G9" t="n">
-        <v>105719</v>
+        <v>91621</v>
       </c>
       <c r="J9" t="n">
         <v>91.5</v>
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>95183</v>
+        <v>83859</v>
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ARC Raiders</t>
+          <t>Limbus Company</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2190,19 +2190,17 @@
           <t>미확인</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
+      <c r="F11" t="n">
+        <v/>
       </c>
       <c r="G11" t="n">
-        <v>80721</v>
+        <v>79143</v>
       </c>
       <c r="J11" t="n">
-        <v>85.2</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="K11" t="n">
-        <v>58900</v>
+        <v/>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -2230,7 +2228,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>76045</v>
+        <v>76446</v>
       </c>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
@@ -2250,7 +2248,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Windrose</t>
+          <t>Delta Force</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -2260,17 +2258,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Action, Adventure, RPG, Early Access</t>
+          <t>Action, Adventure, Massively Multiplayer, Free To Play</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>74455</v>
+        <v>74365</v>
       </c>
       <c r="J13" t="n">
-        <v>87.3</v>
+        <v>58.3</v>
       </c>
       <c r="K13" t="n">
-        <v>32000</v>
+        <v/>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -2282,7 +2280,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Tom Clancy's Rainbow Six Siege</t>
+          <t>ARC Raiders</t>
         </is>
       </c>
       <c r="C14" s="2" t="n"/>
@@ -2294,19 +2292,19 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Action, Free To Play</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>67215</v>
+        <v>68747</v>
       </c>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="n">
-        <v>82.5</v>
+        <v>85.2</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v/>
+        <v>58900</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>0</v>
@@ -2318,7 +2316,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Delta Force</t>
+          <t>Wallpaper Engine</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2328,17 +2326,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Action, Adventure, Massively Multiplayer, Free To Play</t>
+          <t>Casual, Indie, Animation &amp; Modeling, Design &amp; Illustration, Photo Editing, Utilities</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>66122</v>
+        <v>62641</v>
       </c>
       <c r="J15" t="n">
-        <v>58.3</v>
+        <v>98</v>
       </c>
       <c r="K15" t="n">
-        <v/>
+        <v>5600</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -2350,7 +2348,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Wallpaper Engine</t>
+          <t>Windrose</t>
         </is>
       </c>
       <c r="C16" s="2" t="n"/>
@@ -2362,130 +2360,122 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Casual, Indie, Animation &amp; Modeling, Design &amp; Illustration, Photo Editing, Utilities</t>
+          <t>Action, Adventure, RPG, Early Access</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>58572</v>
+        <v>62488</v>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="n">
-        <v>98</v>
+        <v>87.3</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>5600</v>
+        <v>32000</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="A17" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Tom Clancy's Rainbow Six Siege</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Action, Free To Play</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>56454</v>
+      </c>
+      <c r="J17" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="K17" t="n">
+        <v/>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Rust</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>미확인</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Action, Adventure, Indie, Massively Multiplayer, RPG</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>54147</v>
-      </c>
-      <c r="H17" s="4" t="n"/>
-      <c r="I17" s="4" t="n"/>
-      <c r="J17" s="4" t="n">
+      <c r="G18" s="4" t="n">
+        <v>51624</v>
+      </c>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="K17" s="4" t="n">
+      <c r="K18" s="4" t="n">
         <v>21000</v>
       </c>
-      <c r="L17" s="4" t="n">
+      <c r="L18" s="4" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Overwatch®</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>미확인</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Action, Free To Play</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>54073</v>
-      </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n">
-        <v>29.7</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v/>
-      </c>
-      <c r="L18" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
     <row r="19">
-      <c r="A19" s="4" t="n">
+      <c r="A19" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Dead by Daylight</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>미확인</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>52224</v>
-      </c>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n">
-        <v>78.59999999999999</v>
-      </c>
-      <c r="K19" s="4" t="n">
-        <v>8600</v>
-      </c>
-      <c r="L19" s="4" t="n">
-        <v>60</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Warframe</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Action, RPG, Free To Play</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>49756</v>
+      </c>
+      <c r="J19" t="n">
+        <v>87.7</v>
+      </c>
+      <c r="K19" t="n">
+        <v/>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -2494,7 +2484,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Warframe</t>
+          <t>Overwatch®</t>
         </is>
       </c>
       <c r="C20" s="2" t="n"/>
@@ -2506,16 +2496,16 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Action, RPG, Free To Play</t>
+          <t>Action, Free To Play</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>52143</v>
+        <v>48635</v>
       </c>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="n"/>
       <c r="J20" s="2" t="n">
-        <v>87.7</v>
+        <v>29.7</v>
       </c>
       <c r="K20" s="2" t="n">
         <v/>
@@ -2525,35 +2515,39 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Crimson Desert</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>미확인</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Action, Adventure</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>48472</v>
-      </c>
-      <c r="J21" t="n">
-        <v>84</v>
-      </c>
-      <c r="K21" t="n">
-        <v>79800</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Dead by Daylight</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>46769</v>
+      </c>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>8600</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="22">
@@ -2562,7 +2556,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>HELLDIVERS™ 2</t>
+          <t>Crimson Desert</t>
         </is>
       </c>
       <c r="C22" s="2" t="n"/>
@@ -2574,19 +2568,19 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Action, Adventure</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>44924</v>
+        <v>43545</v>
       </c>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="n">
-        <v>76.2</v>
+        <v>84</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>44800</v>
+        <v>79800</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>0</v>
@@ -2598,7 +2592,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Stardew Valley</t>
+          <t>VRChat</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2608,17 +2602,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Indie, RPG, Simulation</t>
+          <t>Adventure, Casual, Massively Multiplayer, Simulation, Sports, Free To Play, Early Access</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>44500</v>
+        <v>43017</v>
       </c>
       <c r="J23" t="n">
-        <v>98.5</v>
+        <v>75.3</v>
       </c>
       <c r="K23" t="n">
-        <v>16000</v>
+        <v/>
       </c>
       <c r="L23" t="n">
         <v>0</v>
@@ -2630,7 +2624,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>VRChat</t>
+          <t>Stardew Valley</t>
         </is>
       </c>
       <c r="C24" s="2" t="n"/>
@@ -2642,19 +2636,19 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Adventure, Casual, Massively Multiplayer, Simulation, Sports, Free To Play, Early Access</t>
+          <t>Indie, RPG, Simulation</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>43861</v>
+        <v>41559</v>
       </c>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n">
-        <v>75.3</v>
+        <v>98.5</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v/>
+        <v>16000</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -2666,7 +2660,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Limbus Company</t>
+          <t>HELLDIVERS™ 2</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2674,17 +2668,19 @@
           <t>미확인</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
       </c>
       <c r="G25" t="n">
-        <v>43573</v>
+        <v>39047</v>
       </c>
       <c r="J25" t="n">
-        <v>87.59999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="K25" t="n">
-        <v/>
+        <v>44800</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -2696,7 +2692,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Geometry Dash</t>
+          <t>Team Fortress 2</t>
         </is>
       </c>
       <c r="C26" s="2" t="n"/>
@@ -2708,19 +2704,19 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Action, Indie</t>
+          <t>Action, Free To Play</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>39322</v>
+        <v>35353</v>
       </c>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n">
-        <v>93.09999999999999</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>5600</v>
+        <v/>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -2732,7 +2728,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Team Fortress 2</t>
+          <t>Geometry Dash</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2742,17 +2738,17 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Action, Free To Play</t>
+          <t>Action, Indie</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>38874</v>
+        <v>33833</v>
       </c>
       <c r="J27" t="n">
-        <v>90.90000000000001</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="K27" t="n">
-        <v/>
+        <v>5600</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -2764,7 +2760,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Baldur's Gate 3</t>
+          <t>War Thunder</t>
         </is>
       </c>
       <c r="C28" s="2" t="n"/>
@@ -2776,19 +2772,19 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Adventure, RPG, Strategy</t>
+          <t>Action, Massively Multiplayer, Simulation, Free To Play</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>34920</v>
+        <v>30342</v>
       </c>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="n">
-        <v>96.8</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>66000</v>
+        <v/>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>

</xml_diff>